<commit_message>
feat(F-NAR-019): ATOM-DIF.ENE.001-07 La grotte bleue
Réécriture vocale example4 : éclat de tapis, énergie vécue.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.ENE.001-07.xlsx
+++ b/stories/arbres/ATOM-DIF.ENE.001-07.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salle de jeux, tapis et tunnel</t>
+          <t>salle de jeux, tapis et tunnel, lampe, rond jaune, grotte de tissu bleu, chaussettes, coussins</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut passer dans le tunnel de tissu. Nino arrive avec beaucoup d'énergie et se met devant. Ils jouent, ils attendent, Nina demande à maman. La grotte frôle les cheveux.</t>
+          <t>Un rond jaune dort sur le tapis. À l'ouverture, un éclat de tapis brille. Nina veut la grotte, maintenant. Nino saute, trop vite. Le tunnel penche. Sourire parti. Elle refuse de foncer. Merci vécu. File des chaussettes, il veut passer. Elle s'arrête, il souffle. Un éclat de tapis tient à l'ouverture.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le tunnel bleu sent le linge propre. Une couture gratte un peu. Nina glisse la main dedans. C'est une grotte. La petite lampe pose un rond jaune sur le tapis. Des chaussettes douces attendent près des coussins. Papa empile deux coussins. La grotte est prête, Nina ? Oui. Elle est bleue. Maman secoue une petite clochette. Ting. Doucement. En ce moment, Nina rampe vers la grotte. Le tapis gratte un peu les genoux. Je veux passer. Dans le tunnel. On fait une file, alors. Nina pose une chaussette près de l'entrée. Elle est chaude, encore. Les chaussures tapent un peu le sol. Nino arrive en sautant. Il a beaucoup d'énergie. Il tourne. Il s'arrête. Il recommence. Il saute, papa. C'est son énergie. Ce n'est pas une faute. Nino se met devant le tunnel. Il a envie d'aller vite. Nina est encore à genoux. Moi aussi, le tunnel. Nino rebondit sur place. Nina regarde maman.</t>
+          <t>Un rond jaune dort sur le tapis. Il est chaud, presque rond. Il est chaud. Tu le vois, Nina ? Oui, papa. La petite lampe pose ce rond, sans bruit. Tes genoux sont sur le tapis, Nina ? Oui, maman. À l'ouverture, un éclat de tapis brille. Il brille, papa. Près du tunnel ? Oui, un petit point. Le tunnel de tissu sent le linge. Une couture gratte un peu, sous les doigts. C'est une grotte. Elle est bleue. La grotte est prête, Nina ? Oui, maman. Papa empile deux coussins, près du tapis. Ils sont mous. Tu les as sentis ? Oui, chauds. Des chaussettes attendent, pliées. Elles sont chaudes, maman. Tu en poses une, près du tissu ? Oui. En ce moment, Nina rampe vers la grotte. Je veux passer, maintenant ! Dans le tunnel, tout de suite. Avec tes genoux ? Oui, papa. Le tapis pique un peu les genoux. Ça pique. Tu glisses la main, Nina ? Oui, maman. Nino arrive près du tapis. Ses chaussures tapent le sol. J'arrive ! Nino ! Il saute sur place, trop vite. Le tunnel ! Moi, le tunnel, maintenant ! Nino se met devant le tissu bleu. Il rebondit, trop près de l'ouverture. Le tunnel penche, un peu. Il penche ! Oh. Nina avance trop, trop vite. Son front touche le tissu, de travers. Je ne passe pas. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Nina ? Oui, papa. Tes mains sont sur le tapis, Nina ? Un peu, maman. L'éclat de tapis tremble, puis tient. Nino rebondit, les pieds légers. Il saute, papa. Nina regarde maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le tunnel bleu sent le linge propre. Une couture gratte un peu. Nina glisse la main dedans. C'est une grotte. La petite lampe pose un rond jaune sur le tapis. Des chaussettes douces attendent près des coussins. Papa empile deux coussins. La grotte est prête, Nina ? Oui. Elle est bleue. Maman secoue une petite clochette. Ting. Doucement. En ce moment, Nina rampe vers la grotte. Le tapis gratte un peu les genoux. Je veux passer. Dans le tunnel. On fait une file, alors. Nina pose une chaussette près de l'entrée. Elle est chaude, encore. Les chaussures tapent un peu le sol. Nino arrive en sautant. Il a beaucoup d'énergie. Il tourne. Il s'arrête. Il recommence. Il saute, papa. C'est son énergie. Ce n'est pas une faute. Nino se met devant le tunnel. Il a envie d'aller vite. Nina est encore à genoux. Moi aussi, le tunnel. Nino rebondit sur place. Nina regarde maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un rond jaune dort sur le tapis. Il est chaud, presque rond. Il est chaud. Tu le vois, Nina ? Oui, papa. La petite lampe pose ce rond, sans bruit. Tes genoux sont sur le tapis, Nina ? Oui, maman. À l'ouverture, un &lt;emphasis level="moderate"&gt;éclat de tapis&lt;/emphasis&gt; brille. Il brille, papa. Près du tunnel ? Oui, un petit point. Le tunnel de tissu sent le linge. Une couture gratte un peu, sous les doigts. C'est une grotte. Elle est bleue. La grotte est prête, Nina ? Oui, maman. Papa empile deux coussins, près du tapis. Ils sont mous. Tu les as sentis ? Oui, chauds. Des chaussettes attendent, pliées. Elles sont chaudes, maman. Tu en poses une, près du tissu ? Oui. En ce moment, Nina rampe vers la grotte. Je veux passer, maintenant ! Dans le tunnel, tout de suite. Avec tes genoux ? Oui, papa. Le tapis pique un peu les genoux. Ça pique. Tu glisses la main, Nina ? Oui, maman. Nino arrive près du tapis. Ses chaussures tapent le sol. J'arrive ! Nino ! Il saute sur place, trop vite. Le tunnel ! Moi, le tunnel, maintenant ! Nino se met devant le tissu bleu. Il rebondit, trop près de l'ouverture. Le tunnel penche, un peu. Il penche ! Oh. Nina avance trop, trop vite. Son front touche le tissu, de travers. Je ne passe pas. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Nina ? Oui, papa. Tes mains sont sur le tapis, Nina ? Un peu, maman. L'éclat de tapis tremble, puis tient. Nino rebondit, les pieds légers. Il saute, papa. Nina regarde maman.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Maman laisse Béatrice dans la salle de jeux. Les chaussures tapent le sol. Ewen arrive en sautant. Il a beaucoup d'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Il tourne. Il s'arrête. Il recommence. Béatrice le regarde. Maman est encore près de la porte. Elle dit : beaucoup d'énergie, ce n'est pas une faute. On peut jouer. On peut attendre. On peut demander à un adulte. Béatrice hoche la tête. Ils font une file pour le tunnel. Ewen a envie d'aller vite. Béatrice dit : on peut attendre. Ewen souffle. Il reste dans la file. Ils jouent. Plus tard, Ewen a encore de l'énergie. Ce n'est pas une faute. Béatrice va vers maman. Elle demande à un adulte. Maman marche avec eux jusqu'aux coussins. On peut jouer ou attendre. Béatrice dit : Ewen a de l'énergie. Maman dit : ce n'est pas une faute. [pause]</t>
+          <t>Un rond jaune dort sur le tapis. Il est chaud, presque rond. Il est chaud. Tu le vois, Nina ? Oui, papa. La petite lampe pose ce rond, sans bruit. Tes genoux sont sur le tapis, Nina ? Oui, maman. À l'ouverture, un &lt;emphasis&gt;éclat de tapis&lt;/emphasis&gt; brille. Il brille, papa. Près du tunnel ? Oui, un petit point. Le tunnel de tissu sent le linge. Une couture gratte un peu, sous les doigts. C'est une grotte. Elle est bleue. La grotte est prête, Nina ? Oui, maman. Papa empile deux coussins, près du tapis. Ils sont mous. Tu les as sentis ? Oui, chauds. Des chaussettes attendent, pliées. Elles sont chaudes, maman. Tu en poses une, près du tissu ? Oui. En ce moment, Nina rampe vers la grotte. Je veux passer, maintenant ! Dans le tunnel, tout de suite. Avec tes genoux ? Oui, papa. Le tapis pique un peu les genoux. Ça pique. Tu glisses la main, Nina ? Oui, maman. Nino arrive près du tapis. Ses chaussures tapent le sol. J'arrive ! Nino ! Il saute sur place, trop vite. Le tunnel ! Moi, le tunnel, maintenant ! Nino se met devant le tissu bleu. Il rebondit, trop près de l'ouverture. Le tunnel penche, un peu. Il penche ! Oh. Nina avance trop, trop vite. Son front touche le tissu, de travers. Je ne passe pas. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Nina ? Oui, papa. Tes mains sont sur le tapis, Nina ? Un peu, maman. L'éclat de tapis tremble, puis tient. Nino rebondit, les pieds légers. Il saute, papa. Nina regarde maman. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>éclat de tapis</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,43 +1321,74 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_grotte_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le tunnel bleu sent le linge propre.
-narrateur|Une couture gratte un peu.
-narrateur|Nina glisse la main dedans.
-narrateur|C'est une grotte.
-narrateur|La petite lampe pose un rond jaune sur le tapis.
-narrateur|Des chaussettes douces attendent près des coussins.
-narrateur|Papa empile deux coussins.
-papa|La grotte est prête, Nina ?
+          <t>narrateur|Un rond jaune dort sur le tapis.
+narrateur|Il est chaud, presque rond.
+enfant-f|Il est chaud.
+papa|Tu le vois, Nina ?
+enfant-f|Oui, papa.
+narrateur|La petite lampe pose ce rond, sans bruit.
+maman|Tes genoux sont sur le tapis, Nina ?
+enfant-f|Oui, maman.
+narrateur|À l'ouverture, un éclat de tapis brille.
+enfant-f|Il brille, papa.
+papa|Près du tunnel ?
+enfant-f|Oui, un petit point.
+narrateur|Le tunnel de tissu sent le linge.
+narrateur|Une couture gratte un peu, sous les doigts.
+enfant-f|C'est une grotte.
+enfant-f|Elle est bleue.
+maman|La grotte est prête, Nina ?
+enfant-f|Oui, maman.
+narrateur|Papa empile deux coussins, près du tapis.
+enfant-f|Ils sont mous.
+papa|Tu les as sentis ?
+enfant-f|Oui, chauds.
+narrateur|Des chaussettes attendent, pliées.
+enfant-f|Elles sont chaudes, maman.
+maman|Tu en poses une, près du tissu ?
 enfant-f|Oui.
-enfant-f|Elle est bleue.
-narrateur|Maman secoue une petite clochette.
-maman|Ting.
-maman|Doucement.
 narrateur|En ce moment, Nina rampe vers la grotte.
-narrateur|Le tapis gratte un peu les genoux.
-enfant-f|Je veux passer.
-enfant-f|Dans le tunnel.
-maman|On fait une file, alors.
-narrateur|Nina pose une chaussette près de l'entrée.
-narrateur|Elle est chaude, encore.
-narrateur|Les chaussures tapent un peu le sol.
-narrateur|Nino arrive en sautant.
-narrateur|Il a beaucoup d'énergie.
-narrateur|Il tourne.
-narrateur|Il s'arrête.
-narrateur|Il recommence.
+enfant-f|Je veux passer, maintenant !
+enfant-f|Dans le tunnel, tout de suite.
+papa|Avec tes genoux ?
+enfant-f|Oui, papa.
+narrateur|Le tapis pique un peu les genoux.
+enfant-f|Ça pique.
+maman|Tu glisses la main, Nina ?
+enfant-f|Oui, maman.
+narrateur|Nino arrive près du tapis.
+narrateur|Ses chaussures tapent le sol.
+copain|J'arrive !
+enfant-f|Nino !
+narrateur|Il saute sur place, trop vite.
+copain|Le tunnel !
+enfant-f|Moi, le tunnel, maintenant !
+narrateur|Nino se met devant le tissu bleu.
+narrateur|Il rebondit, trop près de l'ouverture.
+narrateur|Le tunnel penche, un peu.
+enfant-f|Il penche !
+copain|Oh.
+narrateur|Nina avance trop, trop vite.
+narrateur|Son front touche le tissu, de travers.
+enfant-f|Je ne passe pas.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Nino, Nina ?
+enfant-f|Oui, papa.
+maman|Tes mains sont sur le tapis, Nina ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de tapis tremble, puis tient.
+narrateur|Nino rebondit, les pieds légers.
 enfant-f|Il saute, papa.
-papa|C'est son énergie.
-papa|Ce n'est pas une faute.
-narrateur|Nino se met devant le tunnel.
-narrateur|Il a envie d'aller vite.
-narrateur|Nina est encore à genoux.
-enfant-f|Moi aussi, le tunnel.
-narrateur|Nino rebondit sur place.
 narrateur|Nina regarde maman.</t>
         </is>
       </c>
@@ -1390,12 +1421,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nino a de l'énergie. Que peut-on faire ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino a de l'&lt;emphasis level="moderate"&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Ewen a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1458,18 +1489,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1484,11 +1515,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1499,23 +1530,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1524,23 +1555,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=nino_bouge_trop_vite_que_peut_on_faire; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1573,17 +1604,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina va vers maman. Maman, on fait quoi ? On passe dans la grotte. On attend dans la file. Tu m'as demandé, je t'écoute. On marche jusqu'aux coussins. Maman marche avec eux. Nino s'assoit un moment. Nina s'assoit aussi. Les coussins sont mous et chauds. L'énergie est encore là. Ce n'est pas une faute. On peut attendre. Nino souffle. Il reste dans la file. C'est à Nina. Nina passe dans la grotte. Le tissu frôle ses cheveux. Il est doux. Puis Nino passe. Ils jouent. La clochette fait ting, tout bas. Le tapis est doux sous les mains. On reprend le tunnel après ? Après, oui. Nino pose un coussin. J'attends. Il attend. Nina touche encore le tissu bleu. On y retourne ? Un dernier passage. Nina rampe. Nino attend, les mains sur le coussin. Puis Nino rampe aussi. La clochette, tout doux. Ting.</t>
+          <t>Nina veut le tunnel, tout de suite. Je passe, maintenant ! Elle avance trop vite vers Nino. Les mots se bousculent dans sa bouche. Attends. Nino rebondit, trop près du tissu. Oh. Le sourire ne revient pas. Nina refuse de foncer. Elle referme les mains. Personne ne parle. Elle observe le tunnel, un instant. Elle écoute le tissu qui frôle. Tu veux la grotte avec Nino ? Papa reste à la même hauteur. On va aux coussins ? On marche jusqu'aux coussins ? Oui, maman. Viens, Nino. J'y vais. Ils marchent vers les coussins. Les genoux font un bruit mou. Ils sont mous, papa. Tu t'assois ? Oui. Nina s'assoit un moment. Le tissu du coussin est tiède. Nino s'assoit aussi. Il est tiède. Il souffle. Merci, Nina. Papa a vu les deux, près des coussins. Le tapis est doux, sous les mains. Il est doux. Nino reste, les mains ouvertes. À toi. D'accord. C'est à Nina. Nina rampe dans la grotte. Le tissu frôle ses cheveux. Il est doux. Tu le sens, le bleu ? Oui, papa. Puis Nino passe, sans se presser. J'y vais. Tes cheveux ont frôlé le tissu, Nina ? Oui, maman. Le ventre de Nina se desserre. Les épaules se relèvent un peu. On reste près du tapis ? Oui. Tes genoux sont au chaud ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina va vers maman. Maman, on fait quoi ? On passe dans la grotte. On attend dans la file. Tu m'as demandé, je t'écoute. On marche jusqu'aux coussins. Maman marche avec eux. Nino s'assoit un moment. Nina s'assoit aussi. Les coussins sont mous et chauds. L'énergie est encore là. Ce n'est pas une faute. On peut attendre. Nino souffle. Il reste dans la file. C'est à Nina. Nina passe dans la grotte. Le tissu frôle ses cheveux. Il est doux. Puis Nino passe. Ils jouent. La clochette fait ting, tout bas. Le tapis est doux sous les mains. On reprend le tunnel après ? Après, oui. Nino pose un coussin. J'attends. Il attend. Nina touche encore le tissu bleu. On y retourne ? Un dernier passage. Nina rampe. Nino attend, les mains sur le coussin. Puis Nino rampe aussi. La clochette, tout doux. Ting.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina veut le tunnel, tout de suite. Je passe, maintenant ! Elle avance trop vite vers Nino. Les mots se bousculent dans sa bouche. Attends. Nino rebondit, trop près du tissu. Oh. Le sourire ne revient pas. Nina refuse de foncer. Elle referme les mains. Personne ne parle. Elle observe le tunnel, un instant. Elle écoute le tissu qui frôle. Tu veux la &lt;emphasis level="moderate"&gt;grotte&lt;/emphasis&gt; avec Nino ? Papa reste à la même hauteur. On va aux coussins ? On marche jusqu'aux coussins ? Oui, maman. Viens, Nino. J'y vais. Ils marchent vers les coussins. Les genoux font un bruit mou. Ils sont mous, papa. Tu t'assois ? Oui. Nina s'assoit un moment. Le tissu du coussin est tiède. Nino s'assoit aussi. Il est tiède. Il souffle. Merci, Nina. Papa a vu les deux, près des coussins. Le tapis est doux, sous les mains. Il est doux. Nino reste, les mains ouvertes. À toi. D'accord. C'est à Nina. Nina rampe dans la grotte. Le tissu frôle ses cheveux. Il est doux. Tu le sens, le bleu ? Oui, papa. Puis Nino passe, sans se presser. J'y vais. Tes cheveux ont frôlé le tissu, Nina ? Oui, maman. Le ventre de Nina se desserre. Les épaules se relèvent un peu. On reste près du tapis ? Oui. Tes genoux sont au chaud ? Un peu, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Ewen a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Ce n'est pas une faute. Béatrice a joué. Elle a su attendre. Elle a demandé à un adulte. [pause]</t>
+          <t>Nina veut le tunnel, tout de suite. Je passe, maintenant ! Elle avance trop vite vers Nino. Les mots se bousculent dans sa bouche. Attends. Nino rebondit, trop près du tissu. Oh. Le sourire ne revient pas. Nina refuse de foncer. Elle referme les mains. Personne ne parle. Elle observe le tunnel, un instant. Elle écoute le tissu qui frôle. Tu veux la &lt;emphasis&gt;grotte&lt;/emphasis&gt; avec Nino ? Papa reste à la même hauteur. On va aux coussins ? On marche jusqu'aux coussins ? Oui, maman. Viens, Nino. J'y vais. Ils marchent vers les coussins. Les genoux font un bruit mou. Ils sont mous, papa. Tu t'assois ? Oui. Nina s'assoit un moment. Le tissu du coussin est tiède. Nino s'assoit aussi. Il est tiède. Il souffle. Merci, Nina. Papa a vu les deux, près des coussins. Le tapis est doux, sous les mains. Il est doux. Nino reste, les mains ouvertes. À toi. D'accord. C'est à Nina. Nina rampe dans la grotte. Le tissu frôle ses cheveux. Il est doux. Tu le sens, le bleu ? Oui, papa. Puis Nino passe, sans se presser. J'y vais. Tes cheveux ont frôlé le tissu, Nina ? Oui, maman. Le ventre de Nina se desserre. Les épaules se relèvent un peu. On reste près du tapis ? Oui. Tes genoux sont au chaud ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1630,7 +1661,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1638,10 +1669,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1664,30 +1695,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>grotte</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1696,10 +1727,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1712,47 +1743,64 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_va_aux_coussins_avec_lui; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina va vers maman.
-enfant-f|Maman, on fait quoi ?
-maman|On passe dans la grotte.
-maman|On attend dans la file.
-maman|Tu m'as demandé, je t'écoute.
-maman|On marche jusqu'aux coussins.
-narrateur|Maman marche avec eux.
-narrateur|Nino s'assoit un moment.
-narrateur|Nina s'assoit aussi.
-narrateur|Les coussins sont mous et chauds.
-papa|L'énergie est encore là.
-papa|Ce n'est pas une faute.
-enfant-f|On peut attendre.
-narrateur|Nino souffle.
-narrateur|Il reste dans la file.
+          <t>narrateur|Nina veut le tunnel, tout de suite.
+enfant-f|Je passe, maintenant !
+narrateur|Elle avance trop vite vers Nino.
+narrateur|Les mots se bousculent dans sa bouche.
+copain|Attends.
+narrateur|Nino rebondit, trop près du tissu.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Nina refuse de foncer.
+narrateur|Elle referme les mains.
+narrateur|Personne ne parle.
+narrateur|Elle observe le tunnel, un instant.
+narrateur|Elle écoute le tissu qui frôle.
+papa|Tu veux la grotte avec Nino ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|On va aux coussins ?
+maman|On marche jusqu'aux coussins ?
+enfant-f|Oui, maman.
+papa|Viens, Nino.
+copain|J'y vais.
+narrateur|Ils marchent vers les coussins.
+narrateur|Les genoux font un bruit mou.
+enfant-f|Ils sont mous, papa.
+papa|Tu t'assois ?
+enfant-f|Oui.
+narrateur|Nina s'assoit un moment.
+narrateur|Le tissu du coussin est tiède.
+narrateur|Nino s'assoit aussi.
+copain|Il est tiède.
+narrateur|Il souffle.
+papa|Merci, Nina.
+narrateur|Papa a vu les deux, près des coussins.
+maman|Le tapis est doux, sous les mains.
+enfant-f|Il est doux.
+narrateur|Nino reste, les mains ouvertes.
+copain|À toi.
+enfant-f|D'accord.
 maman|C'est à Nina.
-narrateur|Nina passe dans la grotte.
+narrateur|Nina rampe dans la grotte.
 narrateur|Le tissu frôle ses cheveux.
 enfant-f|Il est doux.
-narrateur|Puis Nino passe.
-narrateur|Ils jouent.
-narrateur|La clochette fait ting, tout bas.
-narrateur|Le tapis est doux sous les mains.
-papa|On reprend le tunnel après ?
-enfant-f|Après, oui.
-narrateur|Nino pose un coussin.
-enfant-m|J'attends.
-narrateur|Il attend.
-narrateur|Nina touche encore le tissu bleu.
-enfant-f|On y retourne ?
-maman|Un dernier passage.
-narrateur|Nina rampe.
-narrateur|Nino attend, les mains sur le coussin.
-narrateur|Puis Nino rampe aussi.
-papa|La clochette, tout doux.
-narrateur|Ting.</t>
+papa|Tu le sens, le bleu ?
+enfant-f|Oui, papa.
+narrateur|Puis Nino passe, sans se presser.
+copain|J'y vais.
+maman|Tes cheveux ont frôlé le tissu, Nina ?
+enfant-f|Oui, maman.
+narrateur|Le ventre de Nina se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près du tapis ?
+enfant-f|Oui.
+maman|Tes genoux sont au chaud ?
+enfant-f|Un peu, maman.</t>
         </is>
       </c>
     </row>
@@ -1779,17 +1827,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On range un coussin ? Oui. Maman prend la main de Nina. Nino range un coussin. La grotte bleue attend demain. La lampe fait encore son rond jaune. J'ai passé. Le tissu a frôlé tes cheveux. Nina plie l'entrée du tunnel. La grotte devient un rectangle bleu.</t>
+          <t>Maman pose des chaussettes près du tapis. Une file, maintenant ! Nino veut passer, trop vite. Il saute vers l'ouverture. Moi d'abord ! Nina avance les mains, trop vite. Puis elle s'arrête net. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le tunnel, un instant. Elle écoute le tissu qui frôle. À l'ouverture, un éclat de tapis luit. Là, sur le tapis. Tu restes, Nino ? Nino ne dit rien. Il souffle, sans parler. Oui. Il reste derrière elle. Une chaussette, maman ? La douce, Nina. Nina pose la chaussette à l'ouverture. Le tissu fait un petit bruit. À moi. Nino pose la sienne, sans se presser. Tu as soufflé, Nino ? Un peu. Le tunnel est droit, Nina ? On passe ? Vous passez ensemble ? Oui, papa. Nina rampe, puis s'arrête un peu. Nino rampe aussi, plus lentement. Le bleu, partout. Le bleu. Le tissu a une poussière, Nina ? Sur le bord.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On range un coussin ? Oui. Maman prend la main de Nina. Nino range un coussin. La grotte bleue attend demain. La lampe fait encore son rond jaune. J'ai passé. Le tissu a frôlé tes cheveux. Nina plie l'entrée du tunnel. La grotte devient un rectangle bleu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman pose des chaussettes près du tapis. Une file, maintenant ! Nino veut passer, trop vite. Il saute vers l'ouverture. Moi d'abord ! Nina avance les mains, trop vite. Puis elle s'arrête net. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le tunnel, un instant. Elle écoute le tissu qui frôle. À l'ouverture, un &lt;emphasis level="moderate"&gt;éclat de tapis&lt;/emphasis&gt; luit. Là, sur le tapis. Tu restes, Nino ? Nino ne dit rien. Il souffle, sans parler. Oui. Il reste derrière elle. Une chaussette, maman ? La douce, Nina. Nina pose la chaussette à l'ouverture. Le tissu fait un petit bruit. À moi. Nino pose la sienne, sans se presser. Tu as soufflé, Nino ? Un peu. Le tunnel est droit, Nina ? On passe ? Vous passez ensemble ? Oui, papa. Nina rampe, puis s'arrête un peu. Nino rampe aussi, plus lentement. Le bleu, partout. Le bleu. Le tissu a une poussière, Nina ? Sur le bord.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman prend la &lt;emphasis&gt;main&lt;/emphasis&gt; de Béatrice. Ewen range un coussin. [pause]</t>
+          <t>Maman pose des chaussettes près du tapis. Une file, maintenant ! Nino veut passer, trop vite. Il saute vers l'ouverture. Moi d'abord ! Nina avance les mains, trop vite. Puis elle s'arrête net. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le tunnel, un instant. Elle écoute le tissu qui frôle. À l'ouverture, un &lt;emphasis&gt;éclat de tapis&lt;/emphasis&gt; luit. Là, sur le tapis. Tu restes, Nino ? Nino ne dit rien. Il souffle, sans parler. Oui. Il reste derrière elle. Une chaussette, maman ? La douce, Nina. Nina pose la chaussette à l'ouverture. Le tissu fait un petit bruit. À moi. Nino pose la sienne, sans se presser. Tu as soufflé, Nino ? Un peu. Le tunnel est droit, Nina ? On passe ? Vous passez ensemble ? Oui, papa. Nina rampe, puis s'arrête un peu. Nino rampe aussi, plus lentement. Le bleu, partout. Le bleu. Le tissu a une poussière, Nina ? Sur le bord. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1836,7 +1884,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1844,10 +1892,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1870,30 +1918,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de tapis</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1902,10 +1950,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1916,19 +1964,50 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_il_souffle_ils_passent; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On range un coussin ?
-enfant-f|Oui.
-narrateur|Maman prend la main de Nina.
-narrateur|Nino range un coussin.
-papa|La grotte bleue attend demain.
-narrateur|La lampe fait encore son rond jaune.
-enfant-f|J'ai passé.
-maman|Le tissu a frôlé tes cheveux.
-narrateur|Nina plie l'entrée du tunnel.
-narrateur|La grotte devient un rectangle bleu.</t>
+          <t>narrateur|Maman pose des chaussettes près du tapis.
+enfant-f|Une file, maintenant !
+narrateur|Nino veut passer, trop vite.
+narrateur|Il saute vers l'ouverture.
+copain|Moi d'abord !
+narrateur|Nina avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le tunnel, un instant.
+narrateur|Elle écoute le tissu qui frôle.
+narrateur|À l'ouverture, un éclat de tapis luit.
+enfant-f|Là, sur le tapis.
+enfant-f|Tu restes, Nino ?
+narrateur|Nino ne dit rien.
+narrateur|Il souffle, sans parler.
+copain|Oui.
+narrateur|Il reste derrière elle.
+enfant-f|Une chaussette, maman ?
+maman|La douce, Nina.
+narrateur|Nina pose la chaussette à l'ouverture.
+narrateur|Le tissu fait un petit bruit.
+copain|À moi.
+narrateur|Nino pose la sienne, sans se presser.
+papa|Tu as soufflé, Nino ?
+copain|Un peu.
+maman|Le tunnel est droit, Nina ?
+enfant-f|On passe ?
+papa|Vous passez ensemble ?
+enfant-f|Oui, papa.
+narrateur|Nina rampe, puis s'arrête un peu.
+narrateur|Nino rampe aussi, plus lentement.
+enfant-f|Le bleu, partout.
+copain|Le bleu.
+maman|Le tissu a une poussière, Nina ?
+enfant-f|Sur le bord.</t>
         </is>
       </c>
     </row>
@@ -1955,17 +2034,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le tunnel bleu est plié. Le rond jaune de la lampe reste. La grotte a été traversée. Deux fois.</t>
+          <t>Ils restent près du tapis. Maman plie un coin du tissu. On a passé, papa. Tu l'as vue, toi ? Oui, la grotte. On est bien, ici. Nina tapote le tissu du doigt. Il est doux, maman. Tu le sens, le bleu ? Oui, maman. Le tunnel est resté, Nina. Oui, avec Nino. Le tunnel est resté. Ça sent le linge, un peu tiède. Et le tapis, maman. Oui, sous les genoux. Les chaussettes restent près du tissu. Un éclat de tapis tient à l'ouverture.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le tunnel bleu est plié. Le rond jaune de la lampe reste. La grotte a été traversée. Deux fois.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du tapis. Maman plie un coin du tissu. On a passé, papa. Tu l'as vue, toi ? Oui, la grotte. On est bien, ici. Nina tapote le tissu du doigt. Il est doux, maman. Tu le sens, le bleu ? Oui, maman. Le tunnel est resté, Nina. Oui, avec Nino. Le tunnel est resté. Ça sent le linge, un peu tiède. Et le tapis, maman. Oui, sous les genoux. Les chaussettes restent près du tissu. Un &lt;emphasis level="moderate"&gt;éclat de tapis&lt;/emphasis&gt; tient à l'ouverture.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du tapis. Maman plie un coin du tissu. On a passé, papa. Tu l'as vue, toi ? Oui, la grotte. On est bien, ici. Nina tapote le tissu du doigt. Il est doux, maman. Tu le sens, le bleu ? Oui, maman. Le tunnel est resté, Nina. Oui, avec Nino. Le tunnel est resté. Ça sent le linge, un peu tiède. Et le tapis, maman. Oui, sous les genoux. Les chaussettes restent près du tissu. Un &lt;emphasis&gt;éclat de tapis&lt;/emphasis&gt; tient à l'ouverture.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2012,18 +2091,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2032,12 +2111,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2046,17 +2125,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de tapis</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2065,11 +2148,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2078,27 +2161,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_a_l_ouverture; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le tunnel bleu est plié.
-narrateur|Le rond jaune de la lampe reste.
-papa|La grotte a été traversée.
-enfant-f|Deux fois.</t>
+          <t>narrateur|Ils restent près du tapis.
+narrateur|Maman plie un coin du tissu.
+enfant-f|On a passé, papa.
+papa|Tu l'as vue, toi ?
+enfant-f|Oui, la grotte.
+maman|On est bien, ici.
+narrateur|Nina tapote le tissu du doigt.
+enfant-f|Il est doux, maman.
+maman|Tu le sens, le bleu ?
+enfant-f|Oui, maman.
+papa|Le tunnel est resté, Nina.
+enfant-f|Oui, avec Nino.
+copain|Le tunnel est resté.
+narrateur|Ça sent le linge, un peu tiède.
+enfant-f|Et le tapis, maman.
+maman|Oui, sous les genoux.
+narrateur|Les chaussettes restent près du tissu.
+narrateur|Un éclat de tapis tient à l'ouverture.</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2204,6 +2305,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>